<commit_message>
add cong no dau ky
</commit_message>
<xml_diff>
--- a/public/bangcongno.xlsx
+++ b/public/bangcongno.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diepm\Desktop\git\diepgia-management\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8266064E-4758-4066-A0F0-CCFC50AE743F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB29E59-79C8-441A-9FAE-9F8F5EA2682D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>BẢNG CÔNG NỢ KHÁCH HÀNG</t>
   </si>
@@ -87,6 +87,12 @@
   </si>
   <si>
     <t>Thời gian</t>
+  </si>
+  <si>
+    <t>Đầu kỳ</t>
+  </si>
+  <si>
+    <t>Tổng</t>
   </si>
 </sst>
 </file>
@@ -178,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -209,6 +215,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -492,26 +501,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O3"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.59765625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.265625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.1328125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="19.86328125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" style="1" customWidth="1"/>
     <col min="5" max="5" width="59" style="1" customWidth="1"/>
-    <col min="6" max="6" width="24.1328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="24.140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="25" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.265625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.86328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.59765625" style="1" customWidth="1"/>
-    <col min="11" max="12" width="13.265625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" style="1" customWidth="1"/>
+    <col min="11" max="12" width="13.28515625" style="1" customWidth="1"/>
     <col min="13" max="13" width="18" style="1" customWidth="1"/>
-    <col min="14" max="14" width="13.1328125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="16.59765625" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.1328125" style="1"/>
+    <col min="14" max="14" width="13.140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="16.5703125" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="45.75" customHeight="1" x14ac:dyDescent="0.8">
+    <row r="1" spans="1:15" ht="45.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -529,13 +538,22 @@
       <c r="M1" s="11"/>
       <c r="N1" s="11"/>
     </row>
-    <row r="2" spans="1:15" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:15" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="5"/>
       <c r="D2" s="4" t="s">
         <v>16</v>
       </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:15" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
@@ -587,7 +605,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2 D2" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>